<commit_message>
First function prototype. fixed GetJsonFromLlm.py json output; previously unable to load json str. updated dri table column for females tab. fully connected all functions together so no inputs are hardcoded.
</commit_message>
<xml_diff>
--- a/DRI_TABLES.xlsx
+++ b/DRI_TABLES.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="37">
   <si>
     <t>age</t>
   </si>
@@ -123,12 +123,6 @@
   </si>
   <si>
     <t>total_water_liters</t>
-  </si>
-  <si>
-    <t>vitamin_d_mg</t>
-  </si>
-  <si>
-    <t>fluoride_mcg</t>
   </si>
 </sst>
 </file>
@@ -1457,113 +1451,113 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="U1" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="X1" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Y1" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="Z1" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="AA1" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="AB1" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="AC1" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="AD1" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="AE1" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="AH1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="AI1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AJ1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="AK1" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="2">

</xml_diff>

<commit_message>
fixed DRI calcualtor accuracy with vitamins; problem orginainted with incorrectly coded DRI_TABLES.xlsx for females and incorrect coding of gui tables.
</commit_message>
<xml_diff>
--- a/DRI_TABLES.xlsx
+++ b/DRI_TABLES.xlsx
@@ -174,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -185,6 +185,9 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1451,91 +1454,91 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="X1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="2" t="s">
+      <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="2" t="s">
+      <c r="AA1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AB1" s="2" t="s">
+      <c r="AB1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="2" t="s">
+      <c r="AC1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AD1" s="2" t="s">
+      <c r="AD1" s="1" t="s">
         <v>29</v>
       </c>
       <c r="AE1" s="1" t="s">
@@ -1556,7 +1559,7 @@
       <c r="AJ1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="2" t="s">
+      <c r="AK1" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1565,12 +1568,12 @@
         <v>1.0</v>
       </c>
       <c r="B2" s="3">
-        <v>1.3</v>
+        <v>300.0</v>
       </c>
       <c r="C2" s="3">
-        <v>300.0</v>
-      </c>
-      <c r="D2" s="3">
+        <v>15.0</v>
+      </c>
+      <c r="D2" s="1">
         <v>15.0</v>
       </c>
       <c r="E2" s="3">
@@ -1580,97 +1583,97 @@
         <v>0.5</v>
       </c>
       <c r="G2" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="H2" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="I2" s="3">
+        <v>0.9</v>
+      </c>
+      <c r="J2" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="K2" s="3">
+        <v>150.0</v>
+      </c>
+      <c r="L2" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="M2" s="3">
+        <v>200.0</v>
+      </c>
+      <c r="N2" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="O2" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="P2" s="3">
+        <v>700.0</v>
+      </c>
+      <c r="Q2" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="R2" s="3">
+        <v>11.0</v>
+      </c>
+      <c r="S2" s="3">
+        <v>340.0</v>
+      </c>
+      <c r="T2" s="3">
+        <v>0.7</v>
+      </c>
+      <c r="U2" s="3">
+        <v>90.0</v>
+      </c>
+      <c r="V2" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="W2" s="3">
+        <v>80.0</v>
+      </c>
+      <c r="X2" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="Y2" s="3">
+        <v>17.0</v>
+      </c>
+      <c r="Z2" s="3">
+        <v>460.0</v>
+      </c>
+      <c r="AA2" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="AB2" s="3">
+        <v>20.0</v>
+      </c>
+      <c r="AC2" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="AD2" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="AE2" s="3">
+        <v>1.05</v>
+      </c>
+      <c r="AF2" s="3">
+        <v>14.0</v>
+      </c>
+      <c r="AG2" s="1">
         <v>30.0</v>
       </c>
-      <c r="H2" s="3">
-        <v>6.0</v>
-      </c>
-      <c r="I2" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="J2" s="3">
-        <v>0.9</v>
-      </c>
-      <c r="K2" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="L2" s="3">
-        <v>150.0</v>
-      </c>
-      <c r="M2" s="3">
-        <v>6.0</v>
-      </c>
-      <c r="N2" s="3">
-        <v>200.0</v>
-      </c>
-      <c r="O2" s="3">
-        <v>2.0</v>
-      </c>
-      <c r="P2" s="3">
-        <v>8.0</v>
-      </c>
-      <c r="Q2" s="3">
-        <v>700.0</v>
-      </c>
-      <c r="R2" s="3">
-        <v>1.5</v>
-      </c>
-      <c r="S2" s="3">
-        <v>11.0</v>
-      </c>
-      <c r="T2" s="3">
-        <v>340.0</v>
-      </c>
-      <c r="U2" s="3">
-        <v>0.7</v>
-      </c>
-      <c r="V2" s="3">
-        <v>90.0</v>
-      </c>
-      <c r="W2" s="3">
-        <v>7.0</v>
-      </c>
-      <c r="X2" s="3">
-        <v>80.0</v>
-      </c>
-      <c r="Y2" s="3">
-        <v>1.2</v>
-      </c>
-      <c r="Z2" s="3">
-        <v>17.0</v>
-      </c>
-      <c r="AA2" s="3">
-        <v>460.0</v>
-      </c>
-      <c r="AB2" s="3">
-        <v>3.0</v>
-      </c>
-      <c r="AC2" s="3">
-        <v>20.0</v>
-      </c>
-      <c r="AD2" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="AE2" s="3">
-        <v>3.0</v>
-      </c>
-      <c r="AF2" s="3">
-        <v>1.05</v>
-      </c>
-      <c r="AG2" s="3">
-        <v>14.0</v>
-      </c>
       <c r="AH2" s="1">
-        <v>30.0</v>
+        <v>40.0</v>
       </c>
       <c r="AI2" s="1">
-        <v>40.0</v>
+        <v>5.0</v>
       </c>
       <c r="AJ2" s="1">
-        <v>5.0</v>
-      </c>
-      <c r="AK2" s="1">
         <v>0.6</v>
+      </c>
+      <c r="AK2" s="3">
+        <v>1.3</v>
       </c>
     </row>
     <row r="3">
@@ -1678,13 +1681,13 @@
         <v>4.0</v>
       </c>
       <c r="B3" s="3">
-        <v>1.7</v>
+        <v>400.0</v>
       </c>
       <c r="C3" s="3">
-        <v>400.0</v>
-      </c>
-      <c r="D3" s="3">
         <v>25.0</v>
+      </c>
+      <c r="D3" s="1">
+        <v>15.0</v>
       </c>
       <c r="E3" s="3">
         <v>0.6</v>
@@ -1693,97 +1696,97 @@
         <v>0.6</v>
       </c>
       <c r="G3" s="3">
-        <v>55.0</v>
+        <v>7.0</v>
       </c>
       <c r="H3" s="3">
-        <v>7.0</v>
+        <v>0.6</v>
       </c>
       <c r="I3" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="J3" s="3">
         <v>0.6</v>
       </c>
-      <c r="J3" s="3">
+      <c r="K3" s="3">
+        <v>200.0</v>
+      </c>
+      <c r="L3" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="M3" s="3">
+        <v>250.0</v>
+      </c>
+      <c r="N3" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="O3" s="3">
+        <v>12.0</v>
+      </c>
+      <c r="P3" s="3">
+        <v>1000.0</v>
+      </c>
+      <c r="Q3" s="3">
+        <v>1.9</v>
+      </c>
+      <c r="R3" s="3">
+        <v>15.0</v>
+      </c>
+      <c r="S3" s="3">
+        <v>440.0</v>
+      </c>
+      <c r="T3" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="U3" s="3">
+        <v>90.0</v>
+      </c>
+      <c r="V3" s="3">
+        <v>10.0</v>
+      </c>
+      <c r="W3" s="3">
+        <v>130.0</v>
+      </c>
+      <c r="X3" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="Y3" s="3">
+        <v>22.0</v>
+      </c>
+      <c r="Z3" s="3">
+        <v>500.0</v>
+      </c>
+      <c r="AA3" s="3">
+        <v>3.8</v>
+      </c>
+      <c r="AB3" s="3">
+        <v>30.0</v>
+      </c>
+      <c r="AC3" s="3">
         <v>1.2</v>
       </c>
-      <c r="K3" s="3">
+      <c r="AD3" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="AE3" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="AF3" s="3">
+        <v>14.0</v>
+      </c>
+      <c r="AG3" s="1">
+        <v>25.0</v>
+      </c>
+      <c r="AH3" s="1">
+        <v>35.0</v>
+      </c>
+      <c r="AI3" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="AJ3" s="1">
         <v>0.6</v>
       </c>
-      <c r="L3" s="3">
-        <v>200.0</v>
-      </c>
-      <c r="M3" s="3">
-        <v>8.0</v>
-      </c>
-      <c r="N3" s="3">
-        <v>250.0</v>
-      </c>
-      <c r="O3" s="3">
-        <v>3.0</v>
-      </c>
-      <c r="P3" s="3">
-        <v>12.0</v>
-      </c>
-      <c r="Q3" s="3">
-        <v>1000.0</v>
-      </c>
-      <c r="R3" s="3">
-        <v>1.9</v>
-      </c>
-      <c r="S3" s="3">
-        <v>15.0</v>
-      </c>
-      <c r="T3" s="3">
-        <v>440.0</v>
-      </c>
-      <c r="U3" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="V3" s="3">
-        <v>90.0</v>
-      </c>
-      <c r="W3" s="3">
-        <v>10.0</v>
-      </c>
-      <c r="X3" s="3">
-        <v>130.0</v>
-      </c>
-      <c r="Y3" s="3">
-        <v>1.5</v>
-      </c>
-      <c r="Z3" s="3">
-        <v>22.0</v>
-      </c>
-      <c r="AA3" s="3">
-        <v>500.0</v>
-      </c>
-      <c r="AB3" s="3">
-        <v>3.8</v>
-      </c>
-      <c r="AC3" s="3">
-        <v>30.0</v>
-      </c>
-      <c r="AD3" s="3">
-        <v>1.2</v>
-      </c>
-      <c r="AE3" s="3">
-        <v>5.0</v>
-      </c>
-      <c r="AF3" s="3">
-        <v>0.95</v>
-      </c>
-      <c r="AG3" s="3">
-        <v>14.0</v>
-      </c>
-      <c r="AH3" s="1">
-        <v>25.0</v>
-      </c>
-      <c r="AI3" s="1">
-        <v>35.0</v>
-      </c>
-      <c r="AJ3" s="1">
-        <v>5.0</v>
-      </c>
-      <c r="AK3" s="1">
-        <v>0.6</v>
+      <c r="AK3" s="3">
+        <v>1.7</v>
       </c>
     </row>
     <row r="4">
@@ -1791,13 +1794,13 @@
         <v>9.0</v>
       </c>
       <c r="B4" s="3">
-        <v>2.1</v>
+        <v>600.0</v>
       </c>
       <c r="C4" s="3">
-        <v>600.0</v>
-      </c>
-      <c r="D4" s="3">
         <v>45.0</v>
+      </c>
+      <c r="D4" s="1">
+        <v>15.0</v>
       </c>
       <c r="E4" s="3">
         <v>1.0</v>
@@ -1806,97 +1809,97 @@
         <v>1.0</v>
       </c>
       <c r="G4" s="3">
-        <v>60.0</v>
+        <v>11.0</v>
       </c>
       <c r="H4" s="3">
-        <v>11.0</v>
+        <v>0.9</v>
       </c>
       <c r="I4" s="3">
+        <v>1.8</v>
+      </c>
+      <c r="J4" s="3">
         <v>0.9</v>
       </c>
-      <c r="J4" s="3">
-        <v>1.8</v>
-      </c>
       <c r="K4" s="3">
-        <v>0.9</v>
+        <v>300.0</v>
       </c>
       <c r="L4" s="3">
-        <v>300.0</v>
+        <v>12.0</v>
       </c>
       <c r="M4" s="3">
-        <v>12.0</v>
+        <v>375.0</v>
       </c>
       <c r="N4" s="3">
-        <v>375.0</v>
+        <v>4.0</v>
       </c>
       <c r="O4" s="3">
-        <v>4.0</v>
+        <v>20.0</v>
       </c>
       <c r="P4" s="3">
+        <v>1300.0</v>
+      </c>
+      <c r="Q4" s="3">
+        <v>2.3</v>
+      </c>
+      <c r="R4" s="3">
+        <v>21.0</v>
+      </c>
+      <c r="S4" s="3">
+        <v>700.0</v>
+      </c>
+      <c r="T4" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="U4" s="3">
+        <v>120.0</v>
+      </c>
+      <c r="V4" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="W4" s="3">
+        <v>240.0</v>
+      </c>
+      <c r="X4" s="3">
+        <v>1.6</v>
+      </c>
+      <c r="Y4" s="3">
+        <v>34.0</v>
+      </c>
+      <c r="Z4" s="3">
+        <v>1250.0</v>
+      </c>
+      <c r="AA4" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="AB4" s="3">
+        <v>40.0</v>
+      </c>
+      <c r="AC4" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="AD4" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="AE4" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="AF4" s="3">
+        <v>14.0</v>
+      </c>
+      <c r="AG4" s="1">
         <v>20.0</v>
       </c>
-      <c r="Q4" s="3">
-        <v>1300.0</v>
-      </c>
-      <c r="R4" s="3">
-        <v>2.3</v>
-      </c>
-      <c r="S4" s="3">
-        <v>21.0</v>
-      </c>
-      <c r="T4" s="3">
-        <v>700.0</v>
-      </c>
-      <c r="U4" s="3">
-        <v>2.0</v>
-      </c>
-      <c r="V4" s="3">
-        <v>120.0</v>
-      </c>
-      <c r="W4" s="3">
-        <v>8.0</v>
-      </c>
-      <c r="X4" s="3">
-        <v>240.0</v>
-      </c>
-      <c r="Y4" s="3">
-        <v>1.6</v>
-      </c>
-      <c r="Z4" s="3">
-        <v>34.0</v>
-      </c>
-      <c r="AA4" s="3">
-        <v>1250.0</v>
-      </c>
-      <c r="AB4" s="3">
-        <v>4.5</v>
-      </c>
-      <c r="AC4" s="3">
-        <v>40.0</v>
-      </c>
-      <c r="AD4" s="3">
-        <v>1.5</v>
-      </c>
-      <c r="AE4" s="3">
-        <v>8.0</v>
-      </c>
-      <c r="AF4" s="3">
-        <v>0.95</v>
-      </c>
-      <c r="AG4" s="3">
-        <v>14.0</v>
-      </c>
       <c r="AH4" s="1">
-        <v>20.0</v>
+        <v>25.0</v>
       </c>
       <c r="AI4" s="1">
-        <v>25.0</v>
+        <v>5.0</v>
       </c>
       <c r="AJ4" s="1">
-        <v>5.0</v>
-      </c>
-      <c r="AK4" s="1">
         <v>0.6</v>
+      </c>
+      <c r="AK4" s="3">
+        <v>2.1</v>
       </c>
     </row>
     <row r="5">
@@ -1904,13 +1907,13 @@
         <v>14.0</v>
       </c>
       <c r="B5" s="3">
-        <v>2.3</v>
+        <v>700.0</v>
       </c>
       <c r="C5" s="3">
-        <v>700.0</v>
-      </c>
-      <c r="D5" s="3">
         <v>65.0</v>
+      </c>
+      <c r="D5" s="1">
+        <v>15.0</v>
       </c>
       <c r="E5" s="3">
         <v>1.2</v>
@@ -1919,97 +1922,97 @@
         <v>1.2</v>
       </c>
       <c r="G5" s="3">
-        <v>75.0</v>
+        <v>15.0</v>
       </c>
       <c r="H5" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="I5" s="3">
+        <v>2.4</v>
+      </c>
+      <c r="J5" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="K5" s="3">
+        <v>400.0</v>
+      </c>
+      <c r="L5" s="3">
+        <v>14.0</v>
+      </c>
+      <c r="M5" s="3">
+        <v>400.0</v>
+      </c>
+      <c r="N5" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="O5" s="3">
+        <v>25.0</v>
+      </c>
+      <c r="P5" s="3">
+        <v>1300.0</v>
+      </c>
+      <c r="Q5" s="3">
+        <v>2.3</v>
+      </c>
+      <c r="R5" s="3">
+        <v>24.0</v>
+      </c>
+      <c r="S5" s="3">
+        <v>890.0</v>
+      </c>
+      <c r="T5" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="U5" s="3">
+        <v>150.0</v>
+      </c>
+      <c r="V5" s="3">
         <v>15.0</v>
       </c>
-      <c r="I5" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="J5" s="3">
-        <v>2.4</v>
-      </c>
-      <c r="K5" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="L5" s="3">
-        <v>400.0</v>
-      </c>
-      <c r="M5" s="3">
+      <c r="W5" s="3">
+        <v>360.0</v>
+      </c>
+      <c r="X5" s="3">
+        <v>1.6</v>
+      </c>
+      <c r="Y5" s="3">
+        <v>43.0</v>
+      </c>
+      <c r="Z5" s="3">
+        <v>1250.0</v>
+      </c>
+      <c r="AA5" s="3">
+        <v>4.7</v>
+      </c>
+      <c r="AB5" s="3">
+        <v>55.0</v>
+      </c>
+      <c r="AC5" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="AD5" s="3">
+        <v>9.0</v>
+      </c>
+      <c r="AE5" s="3">
+        <v>0.85</v>
+      </c>
+      <c r="AF5" s="3">
         <v>14.0</v>
       </c>
-      <c r="N5" s="3">
-        <v>400.0</v>
-      </c>
-      <c r="O5" s="3">
-        <v>5.0</v>
-      </c>
-      <c r="P5" s="3">
+      <c r="AG5" s="1">
+        <v>20.0</v>
+      </c>
+      <c r="AH5" s="1">
         <v>25.0</v>
       </c>
-      <c r="Q5" s="3">
-        <v>1300.0</v>
-      </c>
-      <c r="R5" s="3">
+      <c r="AI5" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="AJ5" s="1">
+        <v>0.6</v>
+      </c>
+      <c r="AK5" s="3">
         <v>2.3</v>
-      </c>
-      <c r="S5" s="3">
-        <v>24.0</v>
-      </c>
-      <c r="T5" s="3">
-        <v>890.0</v>
-      </c>
-      <c r="U5" s="3">
-        <v>3.0</v>
-      </c>
-      <c r="V5" s="3">
-        <v>150.0</v>
-      </c>
-      <c r="W5" s="3">
-        <v>15.0</v>
-      </c>
-      <c r="X5" s="3">
-        <v>360.0</v>
-      </c>
-      <c r="Y5" s="3">
-        <v>1.6</v>
-      </c>
-      <c r="Z5" s="3">
-        <v>43.0</v>
-      </c>
-      <c r="AA5" s="3">
-        <v>1250.0</v>
-      </c>
-      <c r="AB5" s="3">
-        <v>4.7</v>
-      </c>
-      <c r="AC5" s="3">
-        <v>55.0</v>
-      </c>
-      <c r="AD5" s="3">
-        <v>1.5</v>
-      </c>
-      <c r="AE5" s="3">
-        <v>9.0</v>
-      </c>
-      <c r="AF5" s="3">
-        <v>0.85</v>
-      </c>
-      <c r="AG5" s="3">
-        <v>14.0</v>
-      </c>
-      <c r="AH5" s="1">
-        <v>20.0</v>
-      </c>
-      <c r="AI5" s="1">
-        <v>25.0</v>
-      </c>
-      <c r="AJ5" s="1">
-        <v>5.0</v>
-      </c>
-      <c r="AK5" s="1">
-        <v>0.6</v>
       </c>
     </row>
     <row r="6">
@@ -2017,13 +2020,13 @@
         <v>19.0</v>
       </c>
       <c r="B6" s="3">
-        <v>2.7</v>
+        <v>700.0</v>
       </c>
       <c r="C6" s="3">
-        <v>700.0</v>
-      </c>
-      <c r="D6" s="3">
         <v>75.0</v>
+      </c>
+      <c r="D6" s="1">
+        <v>15.0</v>
       </c>
       <c r="E6" s="3">
         <v>1.3</v>
@@ -2032,97 +2035,97 @@
         <v>1.3</v>
       </c>
       <c r="G6" s="3">
-        <v>90.0</v>
+        <v>15.0</v>
       </c>
       <c r="H6" s="3">
-        <v>15.0</v>
+        <v>1.1</v>
       </c>
       <c r="I6" s="3">
+        <v>2.4</v>
+      </c>
+      <c r="J6" s="3">
         <v>1.1</v>
       </c>
-      <c r="J6" s="3">
-        <v>2.4</v>
-      </c>
       <c r="K6" s="3">
-        <v>1.1</v>
+        <v>400.0</v>
       </c>
       <c r="L6" s="3">
-        <v>400.0</v>
+        <v>14.0</v>
       </c>
       <c r="M6" s="3">
+        <v>425.0</v>
+      </c>
+      <c r="N6" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="O6" s="3">
+        <v>30.0</v>
+      </c>
+      <c r="P6" s="3">
+        <v>1000.0</v>
+      </c>
+      <c r="Q6" s="3">
+        <v>2.3</v>
+      </c>
+      <c r="R6" s="3">
+        <v>25.0</v>
+      </c>
+      <c r="S6" s="3">
+        <v>900.0</v>
+      </c>
+      <c r="T6" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="U6" s="3">
+        <v>150.0</v>
+      </c>
+      <c r="V6" s="3">
+        <v>18.0</v>
+      </c>
+      <c r="W6" s="3">
+        <v>310.0</v>
+      </c>
+      <c r="X6" s="3">
+        <v>1.8</v>
+      </c>
+      <c r="Y6" s="3">
+        <v>45.0</v>
+      </c>
+      <c r="Z6" s="3">
+        <v>700.0</v>
+      </c>
+      <c r="AA6" s="3">
+        <v>4.7</v>
+      </c>
+      <c r="AB6" s="3">
+        <v>55.0</v>
+      </c>
+      <c r="AC6" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="AD6" s="3">
+        <v>9.0</v>
+      </c>
+      <c r="AE6" s="3">
+        <v>0.8</v>
+      </c>
+      <c r="AF6" s="3">
         <v>14.0</v>
       </c>
-      <c r="N6" s="3">
-        <v>425.0</v>
-      </c>
-      <c r="O6" s="3">
-        <v>5.0</v>
-      </c>
-      <c r="P6" s="3">
-        <v>30.0</v>
-      </c>
-      <c r="Q6" s="3">
-        <v>1000.0</v>
-      </c>
-      <c r="R6" s="3">
-        <v>2.3</v>
-      </c>
-      <c r="S6" s="3">
+      <c r="AG6" s="1">
+        <v>20.0</v>
+      </c>
+      <c r="AH6" s="1">
         <v>25.0</v>
       </c>
-      <c r="T6" s="3">
-        <v>900.0</v>
-      </c>
-      <c r="U6" s="3">
-        <v>3.0</v>
-      </c>
-      <c r="V6" s="3">
-        <v>150.0</v>
-      </c>
-      <c r="W6" s="3">
-        <v>18.0</v>
-      </c>
-      <c r="X6" s="3">
-        <v>310.0</v>
-      </c>
-      <c r="Y6" s="3">
-        <v>1.8</v>
-      </c>
-      <c r="Z6" s="3">
-        <v>45.0</v>
-      </c>
-      <c r="AA6" s="3">
-        <v>700.0</v>
-      </c>
-      <c r="AB6" s="3">
-        <v>4.7</v>
-      </c>
-      <c r="AC6" s="3">
-        <v>55.0</v>
-      </c>
-      <c r="AD6" s="3">
-        <v>1.5</v>
-      </c>
-      <c r="AE6" s="3">
-        <v>9.0</v>
-      </c>
-      <c r="AF6" s="3">
-        <v>0.8</v>
-      </c>
-      <c r="AG6" s="3">
-        <v>14.0</v>
-      </c>
-      <c r="AH6" s="1">
-        <v>20.0</v>
-      </c>
       <c r="AI6" s="1">
-        <v>25.0</v>
+        <v>5.0</v>
       </c>
       <c r="AJ6" s="1">
-        <v>5.0</v>
-      </c>
-      <c r="AK6" s="1">
         <v>0.6</v>
+      </c>
+      <c r="AK6" s="3">
+        <v>2.7</v>
       </c>
     </row>
     <row r="7">
@@ -2130,13 +2133,13 @@
         <v>31.0</v>
       </c>
       <c r="B7" s="3">
-        <v>2.7</v>
+        <v>700.0</v>
       </c>
       <c r="C7" s="3">
-        <v>700.0</v>
-      </c>
-      <c r="D7" s="3">
         <v>75.0</v>
+      </c>
+      <c r="D7" s="1">
+        <v>15.0</v>
       </c>
       <c r="E7" s="3">
         <v>1.3</v>
@@ -2145,97 +2148,97 @@
         <v>1.3</v>
       </c>
       <c r="G7" s="3">
-        <v>90.0</v>
+        <v>15.0</v>
       </c>
       <c r="H7" s="3">
-        <v>15.0</v>
+        <v>1.1</v>
       </c>
       <c r="I7" s="3">
+        <v>2.4</v>
+      </c>
+      <c r="J7" s="3">
         <v>1.1</v>
       </c>
-      <c r="J7" s="3">
-        <v>2.4</v>
-      </c>
       <c r="K7" s="3">
-        <v>1.1</v>
+        <v>400.0</v>
       </c>
       <c r="L7" s="3">
-        <v>400.0</v>
+        <v>14.0</v>
       </c>
       <c r="M7" s="3">
+        <v>425.0</v>
+      </c>
+      <c r="N7" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="O7" s="3">
+        <v>30.0</v>
+      </c>
+      <c r="P7" s="3">
+        <v>1000.0</v>
+      </c>
+      <c r="Q7" s="3">
+        <v>2.3</v>
+      </c>
+      <c r="R7" s="3">
+        <v>25.0</v>
+      </c>
+      <c r="S7" s="3">
+        <v>900.0</v>
+      </c>
+      <c r="T7" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="U7" s="3">
+        <v>150.0</v>
+      </c>
+      <c r="V7" s="3">
+        <v>18.0</v>
+      </c>
+      <c r="W7" s="3">
+        <v>320.0</v>
+      </c>
+      <c r="X7" s="3">
+        <v>1.8</v>
+      </c>
+      <c r="Y7" s="3">
+        <v>45.0</v>
+      </c>
+      <c r="Z7" s="3">
+        <v>700.0</v>
+      </c>
+      <c r="AA7" s="3">
+        <v>4.7</v>
+      </c>
+      <c r="AB7" s="3">
+        <v>55.0</v>
+      </c>
+      <c r="AC7" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="AD7" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="AE7" s="3">
+        <v>0.8</v>
+      </c>
+      <c r="AF7" s="3">
         <v>14.0</v>
       </c>
-      <c r="N7" s="3">
-        <v>425.0</v>
-      </c>
-      <c r="O7" s="3">
-        <v>5.0</v>
-      </c>
-      <c r="P7" s="3">
-        <v>30.0</v>
-      </c>
-      <c r="Q7" s="3">
-        <v>1000.0</v>
-      </c>
-      <c r="R7" s="3">
-        <v>2.3</v>
-      </c>
-      <c r="S7" s="3">
+      <c r="AG7" s="1">
+        <v>20.0</v>
+      </c>
+      <c r="AH7" s="1">
         <v>25.0</v>
       </c>
-      <c r="T7" s="3">
-        <v>900.0</v>
-      </c>
-      <c r="U7" s="3">
-        <v>3.0</v>
-      </c>
-      <c r="V7" s="3">
-        <v>150.0</v>
-      </c>
-      <c r="W7" s="3">
-        <v>18.0</v>
-      </c>
-      <c r="X7" s="3">
-        <v>320.0</v>
-      </c>
-      <c r="Y7" s="3">
-        <v>1.8</v>
-      </c>
-      <c r="Z7" s="3">
-        <v>45.0</v>
-      </c>
-      <c r="AA7" s="3">
-        <v>700.0</v>
-      </c>
-      <c r="AB7" s="3">
-        <v>4.7</v>
-      </c>
-      <c r="AC7" s="3">
-        <v>55.0</v>
-      </c>
-      <c r="AD7" s="3">
-        <v>1.5</v>
-      </c>
-      <c r="AE7" s="3">
-        <v>8.0</v>
-      </c>
-      <c r="AF7" s="3">
-        <v>0.8</v>
-      </c>
-      <c r="AG7" s="3">
-        <v>14.0</v>
-      </c>
-      <c r="AH7" s="1">
-        <v>20.0</v>
-      </c>
       <c r="AI7" s="1">
-        <v>25.0</v>
+        <v>5.0</v>
       </c>
       <c r="AJ7" s="1">
-        <v>5.0</v>
-      </c>
-      <c r="AK7" s="1">
         <v>0.6</v>
+      </c>
+      <c r="AK7" s="3">
+        <v>2.7</v>
       </c>
     </row>
     <row r="8">
@@ -2243,13 +2246,13 @@
         <v>51.0</v>
       </c>
       <c r="B8" s="3">
-        <v>2.7</v>
+        <v>700.0</v>
       </c>
       <c r="C8" s="3">
-        <v>700.0</v>
-      </c>
-      <c r="D8" s="3">
         <v>75.0</v>
+      </c>
+      <c r="D8" s="1">
+        <v>15.0</v>
       </c>
       <c r="E8" s="3">
         <v>1.5</v>
@@ -2258,97 +2261,97 @@
         <v>1.5</v>
       </c>
       <c r="G8" s="3">
-        <v>90.0</v>
+        <v>15.0</v>
       </c>
       <c r="H8" s="3">
-        <v>15.0</v>
+        <v>1.1</v>
       </c>
       <c r="I8" s="3">
+        <v>2.4</v>
+      </c>
+      <c r="J8" s="3">
         <v>1.1</v>
       </c>
-      <c r="J8" s="3">
-        <v>2.4</v>
-      </c>
       <c r="K8" s="3">
-        <v>1.1</v>
+        <v>400.0</v>
       </c>
       <c r="L8" s="3">
-        <v>400.0</v>
+        <v>14.0</v>
       </c>
       <c r="M8" s="3">
+        <v>425.0</v>
+      </c>
+      <c r="N8" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="O8" s="3">
+        <v>30.0</v>
+      </c>
+      <c r="P8" s="3">
+        <v>1200.0</v>
+      </c>
+      <c r="Q8" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="R8" s="3">
+        <v>20.0</v>
+      </c>
+      <c r="S8" s="3">
+        <v>900.0</v>
+      </c>
+      <c r="T8" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="U8" s="3">
+        <v>150.0</v>
+      </c>
+      <c r="V8" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="W8" s="3">
+        <v>320.0</v>
+      </c>
+      <c r="X8" s="3">
+        <v>1.8</v>
+      </c>
+      <c r="Y8" s="3">
+        <v>45.0</v>
+      </c>
+      <c r="Z8" s="3">
+        <v>700.0</v>
+      </c>
+      <c r="AA8" s="3">
+        <v>4.7</v>
+      </c>
+      <c r="AB8" s="3">
+        <v>55.0</v>
+      </c>
+      <c r="AC8" s="3">
+        <v>1.3</v>
+      </c>
+      <c r="AD8" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="AE8" s="3">
+        <v>0.8</v>
+      </c>
+      <c r="AF8" s="3">
         <v>14.0</v>
       </c>
-      <c r="N8" s="3">
-        <v>425.0</v>
-      </c>
-      <c r="O8" s="3">
-        <v>5.0</v>
-      </c>
-      <c r="P8" s="3">
-        <v>30.0</v>
-      </c>
-      <c r="Q8" s="3">
-        <v>1200.0</v>
-      </c>
-      <c r="R8" s="3">
-        <v>2.0</v>
-      </c>
-      <c r="S8" s="3">
+      <c r="AG8" s="1">
         <v>20.0</v>
       </c>
-      <c r="T8" s="3">
-        <v>900.0</v>
-      </c>
-      <c r="U8" s="3">
-        <v>3.0</v>
-      </c>
-      <c r="V8" s="3">
-        <v>150.0</v>
-      </c>
-      <c r="W8" s="3">
-        <v>8.0</v>
-      </c>
-      <c r="X8" s="3">
-        <v>320.0</v>
-      </c>
-      <c r="Y8" s="3">
-        <v>1.8</v>
-      </c>
-      <c r="Z8" s="3">
-        <v>45.0</v>
-      </c>
-      <c r="AA8" s="3">
-        <v>700.0</v>
-      </c>
-      <c r="AB8" s="3">
-        <v>4.7</v>
-      </c>
-      <c r="AC8" s="3">
-        <v>55.0</v>
-      </c>
-      <c r="AD8" s="3">
-        <v>1.3</v>
-      </c>
-      <c r="AE8" s="3">
-        <v>8.0</v>
-      </c>
-      <c r="AF8" s="3">
-        <v>0.8</v>
-      </c>
-      <c r="AG8" s="3">
-        <v>14.0</v>
-      </c>
       <c r="AH8" s="1">
-        <v>20.0</v>
+        <v>25.0</v>
       </c>
       <c r="AI8" s="1">
-        <v>25.0</v>
+        <v>5.0</v>
       </c>
       <c r="AJ8" s="1">
-        <v>5.0</v>
-      </c>
-      <c r="AK8" s="1">
         <v>0.6</v>
+      </c>
+      <c r="AK8" s="3">
+        <v>2.7</v>
       </c>
     </row>
     <row r="9">
@@ -2356,13 +2359,13 @@
         <v>70.0</v>
       </c>
       <c r="B9" s="3">
-        <v>2.7</v>
+        <v>700.0</v>
       </c>
       <c r="C9" s="3">
-        <v>700.0</v>
-      </c>
-      <c r="D9" s="3">
         <v>75.0</v>
+      </c>
+      <c r="D9" s="1">
+        <v>20.0</v>
       </c>
       <c r="E9" s="3">
         <v>1.5</v>
@@ -2371,98 +2374,122 @@
         <v>1.5</v>
       </c>
       <c r="G9" s="3">
-        <v>90.0</v>
+        <v>15.0</v>
       </c>
       <c r="H9" s="3">
-        <v>15.0</v>
+        <v>1.1</v>
       </c>
       <c r="I9" s="3">
+        <v>2.4</v>
+      </c>
+      <c r="J9" s="3">
         <v>1.1</v>
       </c>
-      <c r="J9" s="3">
-        <v>2.4</v>
-      </c>
       <c r="K9" s="3">
-        <v>1.1</v>
+        <v>400.0</v>
       </c>
       <c r="L9" s="3">
-        <v>400.0</v>
+        <v>14.0</v>
       </c>
       <c r="M9" s="3">
+        <v>425.0</v>
+      </c>
+      <c r="N9" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="O9" s="3">
+        <v>30.0</v>
+      </c>
+      <c r="P9" s="3">
+        <v>1200.0</v>
+      </c>
+      <c r="Q9" s="3">
+        <v>1.8</v>
+      </c>
+      <c r="R9" s="3">
+        <v>20.0</v>
+      </c>
+      <c r="S9" s="3">
+        <v>900.0</v>
+      </c>
+      <c r="T9" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="U9" s="3">
+        <v>150.0</v>
+      </c>
+      <c r="V9" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="W9" s="3">
+        <v>320.0</v>
+      </c>
+      <c r="X9" s="3">
+        <v>1.8</v>
+      </c>
+      <c r="Y9" s="3">
+        <v>45.0</v>
+      </c>
+      <c r="Z9" s="3">
+        <v>700.0</v>
+      </c>
+      <c r="AA9" s="3">
+        <v>4.7</v>
+      </c>
+      <c r="AB9" s="3">
+        <v>55.0</v>
+      </c>
+      <c r="AC9" s="3">
+        <v>1.2</v>
+      </c>
+      <c r="AD9" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="AE9" s="3">
+        <v>0.8</v>
+      </c>
+      <c r="AF9" s="3">
         <v>14.0</v>
       </c>
-      <c r="N9" s="3">
-        <v>425.0</v>
-      </c>
-      <c r="O9" s="3">
-        <v>5.0</v>
-      </c>
-      <c r="P9" s="3">
-        <v>30.0</v>
-      </c>
-      <c r="Q9" s="3">
-        <v>1200.0</v>
-      </c>
-      <c r="R9" s="3">
-        <v>1.8</v>
-      </c>
-      <c r="S9" s="3">
+      <c r="AG9" s="1">
         <v>20.0</v>
       </c>
-      <c r="T9" s="3">
-        <v>900.0</v>
-      </c>
-      <c r="U9" s="3">
-        <v>3.0</v>
-      </c>
-      <c r="V9" s="3">
-        <v>150.0</v>
-      </c>
-      <c r="W9" s="3">
-        <v>8.0</v>
-      </c>
-      <c r="X9" s="3">
-        <v>320.0</v>
-      </c>
-      <c r="Y9" s="3">
-        <v>1.8</v>
-      </c>
-      <c r="Z9" s="3">
-        <v>45.0</v>
-      </c>
-      <c r="AA9" s="3">
-        <v>700.0</v>
-      </c>
-      <c r="AB9" s="3">
-        <v>4.7</v>
-      </c>
-      <c r="AC9" s="3">
-        <v>55.0</v>
-      </c>
-      <c r="AD9" s="3">
-        <v>1.2</v>
-      </c>
-      <c r="AE9" s="3">
-        <v>8.0</v>
-      </c>
-      <c r="AF9" s="3">
-        <v>0.8</v>
-      </c>
-      <c r="AG9" s="3">
-        <v>14.0</v>
-      </c>
       <c r="AH9" s="1">
-        <v>20.0</v>
+        <v>25.0</v>
       </c>
       <c r="AI9" s="1">
-        <v>25.0</v>
+        <v>5.0</v>
       </c>
       <c r="AJ9" s="1">
-        <v>5.0</v>
-      </c>
-      <c r="AK9" s="1">
         <v>0.6</v>
       </c>
+      <c r="AK9" s="3">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="G11" s="4"/>
+    </row>
+    <row r="12">
+      <c r="G12" s="4"/>
+    </row>
+    <row r="13">
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14">
+      <c r="G14" s="4"/>
+    </row>
+    <row r="15">
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16">
+      <c r="G16" s="4"/>
+    </row>
+    <row r="17">
+      <c r="G17" s="4"/>
+    </row>
+    <row r="18">
+      <c r="G18" s="4"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>